<commit_message>
Benchmark \ Data Update
</commit_message>
<xml_diff>
--- a/Minimization Problem with Domain-Induced Discontinuity-Like Behavior/Experimental results/Nonlinear and Discontinuous Function Minimization_Result.xlsx
+++ b/Minimization Problem with Domain-Induced Discontinuity-Like Behavior/Experimental results/Nonlinear and Discontinuous Function Minimization_Result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CPCFile\1stOpt\1stOpt Github\CPC-Benchmark\Minimization Problem with Domain-Induced Discontinuity-Like Behavior\Experimental results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B646854-77AD-4485-8D79-A024E93A337C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7102F361-C0FC-47FE-912E-D04B29652C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="562" firstSheet="26" activeTab="26" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14303" yWindow="-98" windowWidth="19394" windowHeight="11475" tabRatio="562" firstSheet="22" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CPC-DF1" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="889">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="890">
   <si>
     <t>Global Optimal Solution</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2906,6 +2906,10 @@
   </si>
   <si>
     <t>-0.274348422496573</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I,IV</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -13367,7 +13371,7 @@
         <v>194</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -27208,15 +27212,18 @@
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{937908B4-FCA2-496A-86BB-49755C9B2D77}">
-  <dimension ref="A1:XEY30"/>
+  <dimension ref="A1:XEY35"/>
   <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="13.3984375" style="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="10" width="9.8984375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="9.8984375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.59765625" style="13" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="9.8984375" style="13" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.59765625" style="13" bestFit="1" customWidth="1"/>
     <col min="12" max="26" width="11" style="13" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="13.09765625" style="12" bestFit="1" customWidth="1"/>
-    <col min="28" max="31" width="11" style="12" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.3984375" style="12" bestFit="1" customWidth="1"/>
+    <col min="29" max="31" width="11" style="12" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="11" style="11" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="8.8984375" style="11"/>
     <col min="34" max="16384" width="8.8984375" style="25"/>
@@ -27322,7 +27329,7 @@
         <v>388</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>393</v>
+        <v>889</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>388</v>
@@ -27364,7 +27371,7 @@
         <v>776</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>388</v>
@@ -27407,7 +27414,7 @@
       </c>
       <c r="AE3" s="12">
         <f>COUNTIF(B3:Z3, "IV") + COUNTIF(B3:Z3, "II,IV")+COUNTIF(B3:Z3, "I,IV")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:1019 1029:2039 2049:3071 3081:4091 4101:5111 5121:6143 6153:7163 7173:8183 8193:9215 9225:10235 10245:11255 11265:12287 12297:13307 13317:14327 14337:15359 15369:16379">
@@ -32311,6 +32318,12 @@
       <c r="F20" s="5"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="2"/>
@@ -32320,6 +32333,12 @@
       <c r="F21" s="14"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="14"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="25"/>
     </row>
     <row r="22" spans="2:15">
       <c r="B22" s="2"/>
@@ -32329,10 +32348,12 @@
       <c r="F22" s="5"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
-      <c r="N22" s="12"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
     </row>
     <row r="23" spans="2:15">
       <c r="B23" s="2"/>
@@ -32342,7 +32363,12 @@
       <c r="F23" s="14"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
-      <c r="L23" s="29"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="14"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
     </row>
     <row r="24" spans="2:15">
       <c r="B24" s="2"/>
@@ -32352,6 +32378,12 @@
       <c r="F24" s="5"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="2"/>
@@ -32361,6 +32393,12 @@
       <c r="F25" s="14"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="14"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
     </row>
     <row r="26" spans="2:15">
       <c r="B26" s="2"/>
@@ -32370,12 +32408,85 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="5"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="2:15">
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
     </row>
     <row r="28" spans="2:15">
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
       <c r="O28" s="29"/>
     </row>
+    <row r="29" spans="2:15">
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="14"/>
+      <c r="M29" s="25"/>
+      <c r="N29" s="2"/>
+    </row>
     <row r="30" spans="2:15">
-      <c r="L30" s="29"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+    </row>
+    <row r="31" spans="2:15">
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+    </row>
+    <row r="32" spans="2:15">
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
+    </row>
+    <row r="35" spans="8:11">
+      <c r="H35" s="13">
+        <f>H34/49</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="13">
+        <f t="shared" ref="I35:K35" si="8">I34/49</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="13">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="K35" s="13">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>